<commit_message>
fix pressure drop shit
</commit_message>
<xml_diff>
--- a/Pressure drop/fluid_components.xlsx
+++ b/Pressure drop/fluid_components.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Documents\GitHub\PSPL_Rocket_A\Pressure drop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB713677-E2C8-479E-92E8-C6349F1D90DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A38928FC-E66E-4756-BEA3-C5E1343DC995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="37">
   <si>
     <t>Angle [degrees]</t>
   </si>
@@ -55,9 +55,6 @@
     <t>Ball Valve</t>
   </si>
   <si>
-    <t>Fuel</t>
-  </si>
-  <si>
     <t>Bend</t>
   </si>
   <si>
@@ -76,45 +73,15 @@
     <t>LOx Tube 2</t>
   </si>
   <si>
-    <t>LOx Tube to Injector</t>
-  </si>
-  <si>
     <t>LOx Injector Orifices</t>
   </si>
   <si>
     <t>Fuel Tube 1</t>
   </si>
   <si>
-    <t>Fuel Bend 1</t>
-  </si>
-  <si>
     <t>Fuel Tube 2</t>
   </si>
   <si>
-    <t>Fuel Tube 3</t>
-  </si>
-  <si>
-    <t>Fuel Tube 4</t>
-  </si>
-  <si>
-    <t>Fuel Tube 5</t>
-  </si>
-  <si>
-    <t>Fuel Tube 6</t>
-  </si>
-  <si>
-    <t>Fuel Tube 7</t>
-  </si>
-  <si>
-    <t>Fuel Bend 2</t>
-  </si>
-  <si>
-    <t>Fuel Bend 3</t>
-  </si>
-  <si>
-    <t>Fuel Bend 4</t>
-  </si>
-  <si>
     <t>Fuel Run Valve</t>
   </si>
   <si>
@@ -128,13 +95,49 @@
   </si>
   <si>
     <t>Fuel Venturi</t>
+  </si>
+  <si>
+    <t>Oxidizer</t>
+  </si>
+  <si>
+    <t>Fuel Tube to Injector</t>
+  </si>
+  <si>
+    <t>LOx Bend 1</t>
+  </si>
+  <si>
+    <t>LOx Bend 2</t>
+  </si>
+  <si>
+    <t>LOx Tube 3</t>
+  </si>
+  <si>
+    <t>LOx Bend 3</t>
+  </si>
+  <si>
+    <t>LOx Tube 4</t>
+  </si>
+  <si>
+    <t>LOx Bend 4</t>
+  </si>
+  <si>
+    <t>LOx Tube 5</t>
+  </si>
+  <si>
+    <t>LOx Tube 6</t>
+  </si>
+  <si>
+    <t>LOx Tube 7</t>
+  </si>
+  <si>
+    <t>not using venturis!</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -144,6 +147,11 @@
     </font>
     <font>
       <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="26"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -290,13 +298,13 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -616,14 +624,15 @@
     <col min="8" max="8" width="23.1796875" style="2" customWidth="1"/>
     <col min="9" max="9" width="19.54296875" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="30.7265625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>0</v>
@@ -652,7 +661,7 @@
     </row>
     <row r="2" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>8</v>
@@ -673,10 +682,13 @@
       <c r="J2" s="9">
         <v>1E-3</v>
       </c>
+      <c r="L2" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="3" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="L3" s="7" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="M3" s="7" t="s">
         <v>9</v>
@@ -698,7 +710,7 @@
     </row>
     <row r="4" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>8</v>
@@ -722,7 +734,7 @@
     </row>
     <row r="5" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>10</v>
@@ -748,7 +760,7 @@
     </row>
     <row r="6" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>8</v>
@@ -772,10 +784,10 @@
     </row>
     <row r="7" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
@@ -786,9 +798,9 @@
       <c r="I7" s="9"/>
       <c r="J7" s="9"/>
     </row>
-    <row r="8" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:21" ht="34" customHeight="1" x14ac:dyDescent="0.65">
       <c r="A8" s="16" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
@@ -802,7 +814,7 @@
     </row>
     <row r="9" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>8</v>
@@ -826,10 +838,10 @@
     </row>
     <row r="10" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C10" s="12">
         <v>90</v>
@@ -852,7 +864,7 @@
     </row>
     <row r="11" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>8</v>
@@ -879,7 +891,7 @@
         <v>28</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C12" s="12">
         <v>90</v>
@@ -902,7 +914,7 @@
     </row>
     <row r="13" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="10" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>8</v>
@@ -926,10 +938,10 @@
     </row>
     <row r="14" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C14" s="12">
         <v>90</v>
@@ -952,7 +964,7 @@
     </row>
     <row r="15" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="10" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>8</v>
@@ -976,10 +988,10 @@
     </row>
     <row r="16" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="10" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C16" s="12">
         <v>90</v>
@@ -1002,7 +1014,7 @@
     </row>
     <row r="17" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="10" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>8</v>
@@ -1023,10 +1035,13 @@
       <c r="J17" s="11">
         <v>1E-3</v>
       </c>
+      <c r="L17" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="18" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="L18" s="10" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="M18" s="10" t="s">
         <v>9</v>
@@ -1048,7 +1063,7 @@
     </row>
     <row r="19" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="10" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B19" s="10" t="s">
         <v>8</v>
@@ -1072,7 +1087,7 @@
     </row>
     <row r="20" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="10" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>10</v>
@@ -1098,7 +1113,7 @@
     </row>
     <row r="21" spans="1:21" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="10" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>8</v>
@@ -1122,10 +1137,10 @@
     </row>
     <row r="22" spans="1:21" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A22" s="10" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C22" s="11"/>
       <c r="D22" s="11"/>

</xml_diff>